<commit_message>
Add SKU Excel import and category-aware marketplace mapping
</commit_message>
<xml_diff>
--- a/Пример для автозагрузки.xlsx
+++ b/Пример для автозагрузки.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/konstantin/Documents/Codex/Codex Проекты/Калькулятор PIM.Seller/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37097E5C-C9A2-0E48-A321-4034F7D3314A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E097FD-1A4B-D546-A43A-B2B02034EFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3880" yWindow="3000" windowWidth="22280" windowHeight="12460" xr2:uid="{C58084C8-A65E-EE41-9274-78CFD50C4A6E}"/>
+    <workbookView xWindow="1240" yWindow="3000" windowWidth="22280" windowHeight="12460" xr2:uid="{C58084C8-A65E-EE41-9274-78CFD50C4A6E}"/>
   </bookViews>
   <sheets>
     <sheet name="ВГХ" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,13 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>ВГХ товаров</t>
-  </si>
-  <si>
-    <t>Артикул</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>вес</t>
   </si>
@@ -59,16 +54,43 @@
     <t>ширина</t>
   </si>
   <si>
-    <t>объемный вес</t>
-  </si>
-  <si>
-    <t>Фитнес браслет Smart Band 9 Active</t>
-  </si>
-  <si>
-    <t>https://www.wildberries.ru/catalog/280589425/detail.aspx?targetUrl=GP</t>
-  </si>
-  <si>
     <t>Наименование</t>
+  </si>
+  <si>
+    <t>штук на паллете</t>
+  </si>
+  <si>
+    <t>Ссылка на товар WB</t>
+  </si>
+  <si>
+    <t>Ссылка на товар OZON</t>
+  </si>
+  <si>
+    <t>Миксер кухонный</t>
+  </si>
+  <si>
+    <t>https://www.wildberries.ru/catalog/584775688/detail.aspx</t>
+  </si>
+  <si>
+    <t>https://www.ozon.ru/product/planetarnyy-mikser-elektricheskiy-kuhonnyy-4-v-1-kitfort-kt-4419-3044450223/?at=oZt6RxGZMumBJq5WSwPgn3kI6BRQQ5tDVRw6rf9LLq5B</t>
+  </si>
+  <si>
+    <t>Тип товара Ozon</t>
+  </si>
+  <si>
+    <t>WB пердмет</t>
+  </si>
+  <si>
+    <t>Миксеры</t>
+  </si>
+  <si>
+    <t>Характеристики товаров</t>
+  </si>
+  <si>
+    <t>Планетарный миксер</t>
+  </si>
+  <si>
+    <t>Цена с НДС</t>
   </si>
 </sst>
 </file>
@@ -78,7 +100,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -135,22 +157,35 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -253,6 +288,155 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -269,68 +453,111 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -548,203 +775,338 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{926CE9DD-53AC-854B-8FBD-336B22106F61}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="B1:L31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="2" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="2:12" ht="14" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+    </row>
+    <row r="2" spans="2:12" ht="31" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.15">
-      <c r="A2" s="3" t="s">
+      <c r="I2" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" s="19" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="34">
+        <v>15034</v>
+      </c>
+      <c r="D3" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="11" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="E3" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="8">
-        <v>0.09</v>
-      </c>
-      <c r="D3" s="9">
-        <v>10</v>
-      </c>
-      <c r="E3" s="9">
-        <v>3</v>
-      </c>
-      <c r="F3" s="9">
-        <v>10</v>
-      </c>
-      <c r="G3" s="10">
-        <f t="shared" ref="G3:G6" si="0">D3*E3*F3/5000</f>
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="10"/>
-    </row>
-    <row r="5" spans="1:7" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="10"/>
-    </row>
-    <row r="6" spans="1:7" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
+      <c r="H3" s="26">
+        <v>9.42</v>
+      </c>
+      <c r="I3" s="27">
+        <v>30.8</v>
+      </c>
+      <c r="J3" s="27">
+        <v>60</v>
+      </c>
+      <c r="K3" s="27">
+        <v>39.6</v>
+      </c>
+      <c r="L3" s="28">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B4" s="1"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="23"/>
+    </row>
+    <row r="5" spans="2:12" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B5" s="1"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="23"/>
+    </row>
+    <row r="6" spans="2:12" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="6"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
       <c r="G6" s="17"/>
-    </row>
-    <row r="7" spans="1:7" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-    </row>
-    <row r="8" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-    </row>
-    <row r="9" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-    </row>
-    <row r="10" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-    </row>
-    <row r="11" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-    </row>
-    <row r="12" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-    </row>
-    <row r="13" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-    </row>
-    <row r="14" spans="1:7" s="19" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-    </row>
-    <row r="15" spans="1:7" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-    </row>
-    <row r="16" spans="1:7" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-    </row>
-    <row r="17" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-    </row>
-    <row r="18" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A18" s="20"/>
-      <c r="B18" s="20"/>
-    </row>
-    <row r="19" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-    </row>
-    <row r="20" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-    </row>
-    <row r="21" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A21" s="20"/>
-      <c r="B21" s="20"/>
-    </row>
-    <row r="22" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-    </row>
-    <row r="23" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-    </row>
-    <row r="24" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A24" s="20"/>
-      <c r="B24" s="20"/>
-    </row>
-    <row r="25" spans="1:2" s="11" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A26" s="21"/>
-      <c r="B26" s="21"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A28" s="21"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A29" s="21"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A30" s="21"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A31" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="24"/>
+    </row>
+    <row r="7" spans="2:12" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="2:12" s="10" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="2:12" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+    </row>
+    <row r="16" spans="2:12" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+    </row>
+    <row r="17" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+    </row>
+    <row r="18" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+    </row>
+    <row r="20" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+    </row>
+    <row r="21" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+    </row>
+    <row r="22" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+    </row>
+    <row r="24" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+    </row>
+    <row r="25" spans="2:7" s="4" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.15">
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B1:L1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{02DD74B6-DB68-D34F-ADC0-FD783C6496A4}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2478677F-4AC8-5040-BF0B-55C3C8E33433}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>